<commit_message>
changes may 16 -1
</commit_message>
<xml_diff>
--- a/TestData/LV_T1624_OpportunityToEngagementConversionMappingForFRJobTypes.xlsx
+++ b/TestData/LV_T1624_OpportunityToEngagementConversionMappingForFRJobTypes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE7EA8F5-7562-4E9E-97F0-6C9EB15D943C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F02274-6930-45C2-824C-03C105F0E6F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AddOpportunity" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="89">
   <si>
     <t>Client</t>
   </si>
@@ -294,6 +294,9 @@
   </si>
   <si>
     <t>Chris1 Lord1</t>
+  </si>
+  <si>
+    <t>Andy Chen</t>
   </si>
 </sst>
 </file>
@@ -1022,37 +1025,37 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AF9"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="14.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.5546875" style="4" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="21" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="27" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="11" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" customWidth="1"/>
-    <col min="29" max="29" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.33203125" customWidth="1"/>
+    <col min="29" max="29" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1150,7 +1153,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>73</v>
       </c>
@@ -1191,7 +1194,7 @@
         <v>16</v>
       </c>
       <c r="N2" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>85</v>
@@ -1248,7 +1251,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -1289,7 +1292,7 @@
         <v>16</v>
       </c>
       <c r="N3" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="O3" s="3" t="s">
         <v>85</v>
@@ -1346,7 +1349,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>73</v>
       </c>
@@ -1387,7 +1390,7 @@
         <v>16</v>
       </c>
       <c r="N4" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="O4" s="3" t="s">
         <v>85</v>
@@ -1444,7 +1447,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>73</v>
       </c>
@@ -1485,7 +1488,7 @@
         <v>16</v>
       </c>
       <c r="N5" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="O5" s="3" t="s">
         <v>85</v>
@@ -1542,7 +1545,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>73</v>
       </c>
@@ -1583,7 +1586,7 @@
         <v>16</v>
       </c>
       <c r="N6" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="O6" s="3" t="s">
         <v>85</v>
@@ -1640,7 +1643,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>73</v>
       </c>
@@ -1681,7 +1684,7 @@
         <v>16</v>
       </c>
       <c r="N7" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="O7" s="3" t="s">
         <v>85</v>
@@ -1738,7 +1741,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>73</v>
       </c>
@@ -1779,7 +1782,7 @@
         <v>16</v>
       </c>
       <c r="N8" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="O8" s="3" t="s">
         <v>85</v>
@@ -1836,7 +1839,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>73</v>
       </c>
@@ -1877,7 +1880,7 @@
         <v>16</v>
       </c>
       <c r="N9" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="O9" s="3" t="s">
         <v>85</v>
@@ -1944,14 +1947,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -1962,7 +1965,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>81</v>
       </c>
@@ -1982,14 +1985,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19F56F96-8E69-465C-AD2C-16F74E4333CC}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>78</v>
       </c>
@@ -2002,17 +2005,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32A82162-87C2-47FB-939D-25F1C99EC756}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>80</v>
       </c>
@@ -2025,17 +2028,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
@@ -2061,7 +2064,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>87</v>
       </c>
@@ -2096,14 +2099,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" customWidth="1"/>
-    <col min="4" max="4" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" customWidth="1"/>
+    <col min="4" max="4" width="29.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>52</v>
       </c>
@@ -2117,7 +2120,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>69</v>
       </c>
@@ -2131,7 +2134,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>69</v>
       </c>
@@ -2145,7 +2148,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>69</v>
       </c>
@@ -2159,7 +2162,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>69</v>
       </c>
@@ -2173,7 +2176,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>69</v>
       </c>
@@ -2187,7 +2190,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>69</v>
       </c>
@@ -2201,7 +2204,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>69</v>
       </c>
@@ -2215,7 +2218,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>69</v>
       </c>

</xml_diff>

<commit_message>
User changes May 17 24 -1
</commit_message>
<xml_diff>
--- a/TestData/LV_T1624_OpportunityToEngagementConversionMappingForFRJobTypes.xlsx
+++ b/TestData/LV_T1624_OpportunityToEngagementConversionMappingForFRJobTypes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F96F4734-0EB5-41DC-8485-2D5AD22CAC56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40EC4FBA-7F4A-46BF-A2A4-D73CB627B683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="89">
   <si>
     <t>Client</t>
   </si>
@@ -1024,7 +1024,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AF9"/>
+  <dimension ref="A1:AF8"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
@@ -1162,8 +1162,8 @@
       <c r="B2" t="s">
         <v>73</v>
       </c>
-      <c r="C2" s="7" t="s">
-        <v>57</v>
+      <c r="C2" s="5" t="s">
+        <v>58</v>
       </c>
       <c r="D2" t="s">
         <v>86</v>
@@ -1250,7 +1250,7 @@
         <v>8</v>
       </c>
       <c r="AF2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.3">
@@ -1260,8 +1260,8 @@
       <c r="B3" t="s">
         <v>73</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>58</v>
+      <c r="C3" t="s">
+        <v>59</v>
       </c>
       <c r="D3" t="s">
         <v>86</v>
@@ -1348,7 +1348,7 @@
         <v>8</v>
       </c>
       <c r="AF3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.3">
@@ -1359,7 +1359,7 @@
         <v>73</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D4" t="s">
         <v>86</v>
@@ -1446,7 +1446,7 @@
         <v>8</v>
       </c>
       <c r="AF4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.3">
@@ -1457,7 +1457,7 @@
         <v>73</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
         <v>86</v>
@@ -1544,7 +1544,7 @@
         <v>8</v>
       </c>
       <c r="AF5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.3">
@@ -1555,7 +1555,7 @@
         <v>73</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D6" t="s">
         <v>86</v>
@@ -1642,7 +1642,7 @@
         <v>8</v>
       </c>
       <c r="AF6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.3">
@@ -1653,7 +1653,7 @@
         <v>73</v>
       </c>
       <c r="C7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D7" t="s">
         <v>86</v>
@@ -1740,7 +1740,7 @@
         <v>8</v>
       </c>
       <c r="AF7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.3">
@@ -1751,7 +1751,7 @@
         <v>73</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D8" t="s">
         <v>86</v>
@@ -1838,104 +1838,6 @@
         <v>8</v>
       </c>
       <c r="AF8" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>73</v>
-      </c>
-      <c r="B9" t="s">
-        <v>73</v>
-      </c>
-      <c r="C9" t="s">
-        <v>64</v>
-      </c>
-      <c r="D9" t="s">
-        <v>86</v>
-      </c>
-      <c r="E9" t="s">
-        <v>7</v>
-      </c>
-      <c r="F9" t="s">
-        <v>8</v>
-      </c>
-      <c r="G9" t="s">
-        <v>8</v>
-      </c>
-      <c r="H9" t="s">
-        <v>11</v>
-      </c>
-      <c r="I9" t="s">
-        <v>8</v>
-      </c>
-      <c r="J9" t="s">
-        <v>8</v>
-      </c>
-      <c r="K9" t="s">
-        <v>83</v>
-      </c>
-      <c r="L9" t="s">
-        <v>71</v>
-      </c>
-      <c r="M9" t="s">
-        <v>16</v>
-      </c>
-      <c r="N9" t="s">
-        <v>88</v>
-      </c>
-      <c r="O9" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="P9" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q9" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="R9" t="s">
-        <v>25</v>
-      </c>
-      <c r="S9" t="s">
-        <v>25</v>
-      </c>
-      <c r="T9" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="U9" t="s">
-        <v>28</v>
-      </c>
-      <c r="V9" t="s">
-        <v>72</v>
-      </c>
-      <c r="W9" t="s">
-        <v>31</v>
-      </c>
-      <c r="X9" t="s">
-        <v>33</v>
-      </c>
-      <c r="Y9" t="s">
-        <v>56</v>
-      </c>
-      <c r="Z9" t="s">
-        <v>40</v>
-      </c>
-      <c r="AA9" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="AB9" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="AC9" t="s">
-        <v>66</v>
-      </c>
-      <c r="AD9" t="s">
-        <v>8</v>
-      </c>
-      <c r="AE9" t="s">
-        <v>8</v>
-      </c>
-      <c r="AF9" t="s">
         <v>75</v>
       </c>
     </row>

</xml_diff>

<commit_message>
FR ERP Status 5-19-2025
</commit_message>
<xml_diff>
--- a/TestData/LV_T1624_OpportunityToEngagementConversionMappingForFRJobTypes.xlsx
+++ b/TestData/LV_T1624_OpportunityToEngagementConversionMappingForFRJobTypes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39372AE4-CF94-466C-A891-E1457481499F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D1AAB3-F40D-4ED9-BAC0-54F116DCFA38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AddOpportunity" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="99">
   <si>
     <t>Client</t>
   </si>
@@ -323,6 +323,12 @@
   </si>
   <si>
     <t>Legal Hold test Notes</t>
+  </si>
+  <si>
+    <t>Ajay Nair</t>
+  </si>
+  <si>
+    <t>System Admin</t>
   </si>
 </sst>
 </file>
@@ -1914,7 +1920,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7AA2166-0BC1-42EB-8C55-F0979EE9638D}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
@@ -1942,6 +1948,14 @@
       </c>
       <c r="B3" t="s">
         <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes June 4 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_T1624_OpportunityToEngagementConversionMappingForFRJobTypes.xlsx
+++ b/TestData/LV_T1624_OpportunityToEngagementConversionMappingForFRJobTypes.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D1AAB3-F40D-4ED9-BAC0-54F116DCFA38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABAB4B98-4460-4A50-A0A4-D2A4CECCE770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="AddOpportunity" sheetId="1" r:id="rId1"/>
-    <sheet name="Users" sheetId="2" r:id="rId2"/>
-    <sheet name="CAOUser" sheetId="8" r:id="rId3"/>
-    <sheet name="AppName" sheetId="5" r:id="rId4"/>
-    <sheet name="ModuleName" sheetId="6" r:id="rId5"/>
+    <sheet name="Users" sheetId="2" r:id="rId1"/>
+    <sheet name="CAOUser" sheetId="8" r:id="rId2"/>
+    <sheet name="AppName" sheetId="5" r:id="rId3"/>
+    <sheet name="ModuleName" sheetId="6" r:id="rId4"/>
+    <sheet name="AddOpportunity" sheetId="1" r:id="rId5"/>
     <sheet name="AddContact" sheetId="3" r:id="rId6"/>
     <sheet name="Engagement" sheetId="4" r:id="rId7"/>
     <sheet name="Notes" sheetId="7" r:id="rId8"/>
@@ -1055,41 +1055,172 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7AA2166-0BC1-42EB-8C55-F0979EE9638D}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19F56F96-8E69-465C-AD2C-16F74E4333CC}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32A82162-87C2-47FB-939D-25F1C99EC756}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AF8"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.44140625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="8" style="4" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="21" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="27" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="11" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" customWidth="1"/>
-    <col min="29" max="29" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.33203125" customWidth="1"/>
+    <col min="29" max="29" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1187,7 +1318,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>71</v>
       </c>
@@ -1285,7 +1416,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -1383,7 +1514,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>71</v>
       </c>
@@ -1481,7 +1612,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -1579,7 +1710,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>71</v>
       </c>
@@ -1677,7 +1808,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>71</v>
       </c>
@@ -1775,7 +1906,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>71</v>
       </c>
@@ -1880,151 +2011,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>79</v>
-      </c>
-      <c r="B2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7AA2166-0BC1-42EB-8C55-F0979EE9638D}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19F56F96-8E69-465C-AD2C-16F74E4333CC}">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32A82162-87C2-47FB-939D-25F1C99EC756}">
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>32</v>
       </c>
@@ -2050,7 +2050,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>70</v>
       </c>
@@ -2085,14 +2085,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" customWidth="1"/>
-    <col min="4" max="4" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" customWidth="1"/>
+    <col min="4" max="4" width="29.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>50</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>67</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>67</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>67</v>
       </c>
@@ -2148,7 +2148,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>67</v>
       </c>
@@ -2162,7 +2162,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>67</v>
       </c>
@@ -2176,7 +2176,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>67</v>
       </c>
@@ -2190,7 +2190,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>67</v>
       </c>
@@ -2204,7 +2204,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>67</v>
       </c>
@@ -2227,17 +2227,17 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{388A5FB4-80B0-4A36-B46C-8E2770C1F8E1}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>96</v>
       </c>

</xml_diff>